<commit_message>
Beta feedback template — Andreas review edits
Three changes from Andreas's reviewed copy
(beta_feedback_template_aw.xlsx):

1. Instructions R7 (Correction definition): append
   " or not IPCC-compliant" to broaden the category.

2. Instructions R9 (General definition): append
   ", or feedback from user experience such as a challenge that you
   were later able to overcome" so reviewers know to log learning
   experiences, not just questions.

3. Type_definitions sheet column order:
   Type | Severity | Type_def | Sev_def
                  →
   Type | Type_def | Severity | Sev_def

   First two columns are now the category (Type + its definition);
   last two are severity (Severity + its definition) — easier to
   read than the previous interleaved layout.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/beta_feedback_template.xlsx
+++ b/beta_feedback_template.xlsx
@@ -1,184 +1,177 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cgiar.sharepoint.com/sites/Alliance-ClimateActionNetZero/Shared Documents/ClimateActionNetZero/1_Projects/D614 _GMH_Emissions_Uncertainty/2_Technical_&amp;_Data/cattle-uncertainty-app/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_7193DAA9B3F863125E9572328B6465C39281B919" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookPr date1904="false"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="380" windowWidth="14400" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Instructions" sheetId="1" r:id="rId1"/>
-    <sheet name="Feedback" sheetId="2" r:id="rId2"/>
-    <sheet name="Type_definitions" sheetId="3" r:id="rId3"/>
+    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Feedback" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Type_definitions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="50">
-  <si>
-    <t>IPCC Tier 2 Livestock GHG Uncertainty Calculator — Beta Testing Feedback Form</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>HOW TO USE THIS TEMPLATE</t>
-  </si>
-  <si>
-    <t>1. Fill in one row per comment in the 'Feedback' sheet.</t>
-  </si>
-  <si>
-    <t>2. Use the Type dropdown to classify your comment:</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+  <si>
+    <t xml:space="preserve">IPCC Tier 2 Livestock GHG Uncertainty Calculator — Beta Testing Feedback Form</t>
+  </si>
+  <si>
+    <t xml:space="preserve"/>
+  </si>
+  <si>
+    <t xml:space="preserve">HOW TO USE THIS TEMPLATE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Fill in one row per comment in the 'Feedback' sheet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Use the Type dropdown to classify your comment:</t>
   </si>
   <si>
     <t xml:space="preserve">   Bug          — the tool crashes, produces wrong numbers, or behaves unexpectedly</t>
   </si>
   <si>
-    <t xml:space="preserve">   Correction   — something is factually incorrect (method, equation, reference)</t>
+    <t xml:space="preserve">   Correction   — something is factually incorrect (method, equation, reference) or not IPCC-compliant</t>
   </si>
   <si>
     <t xml:space="preserve">   Enhancement  — a feature that would make the tool more useful</t>
   </si>
   <si>
-    <t xml:space="preserve">   General      — a general comment or question</t>
-  </si>
-  <si>
-    <t>3. Use Severity to indicate urgency (Critical = must fix before release).</t>
-  </si>
-  <si>
-    <t>4. In 'Suggested fix', note the expected behaviour or your proposed solution.</t>
-  </si>
-  <si>
-    <t>5. Save your completed file and email it to lolita.muller26@gmail.com.</t>
-  </si>
-  <si>
-    <t>6. Multiple reviewers: combine sheets by appending rows — the Reviewer name column keeps them distinct.</t>
-  </si>
-  <si>
-    <t>COLUMN DEFINITIONS</t>
-  </si>
-  <si>
-    <t>Reviewer name   — Your full name</t>
-  </si>
-  <si>
-    <t>Date            — Date of the observation (YYYY-MM-DD)</t>
-  </si>
-  <si>
-    <t>Tab             — Which app tab (Home, Data Input, QA/QC, Uncertainty, Correlations, Simulate, Sensitivity, IPCC Report, Resources, Definitions)</t>
-  </si>
-  <si>
-    <t>Screen element  — The specific button, table, chart, or text that the comment relates to</t>
-  </si>
-  <si>
-    <t>Type            — Bug / Correction / Enhancement / General</t>
-  </si>
-  <si>
-    <t>Severity        — Critical / High / Medium / Low</t>
-  </si>
-  <si>
-    <t>Description     — What you observed or what the problem is</t>
-  </si>
-  <si>
-    <t>Suggested fix   — What the correct behaviour should be, or your proposed solution</t>
-  </si>
-  <si>
-    <t>Status          — Leave blank; will be filled by the development team</t>
-  </si>
-  <si>
-    <t>Reviewer name</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Tab</t>
-  </si>
-  <si>
-    <t>Screen element / feature</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>Severity</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Suggested fix / comment</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Type_def</t>
-  </si>
-  <si>
-    <t>Sev_def</t>
-  </si>
-  <si>
-    <t>Bug</t>
-  </si>
-  <si>
-    <t>Critical</t>
-  </si>
-  <si>
-    <t>The tool crashes, produces wrong output, or behaves unexpectedly</t>
-  </si>
-  <si>
-    <t>Must fix before any external release — calculation error or crash</t>
-  </si>
-  <si>
-    <t>Correction</t>
-  </si>
-  <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>Something is factually incorrect — wrong equation, wrong IPCC reference, wrong number</t>
-  </si>
-  <si>
-    <t>Should fix before external release — significant usability or accuracy issue</t>
-  </si>
-  <si>
-    <t>Enhancement</t>
-  </si>
-  <si>
-    <t>Medium</t>
-  </si>
-  <si>
-    <t>A feature that would make the tool more useful or easier to use</t>
-  </si>
-  <si>
-    <t>Can fix in next iteration — minor issue that does not block use</t>
-  </si>
-  <si>
-    <t>General</t>
-  </si>
-  <si>
-    <t>Low</t>
-  </si>
-  <si>
-    <t>A general observation, question, or comment</t>
-  </si>
-  <si>
-    <t>Nice to have — cosmetic or very minor improvement</t>
+    <t xml:space="preserve">   General      — a general comment or question, or feedback from user experience such as a challenge that you were later able to overcome</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Use Severity to indicate urgency (Critical = must fix before release).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. In 'Suggested fix', note the expected behaviour or your proposed solution.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Save your completed file and email it to lolita.muller26@gmail.com.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Multiple reviewers: combine sheets by appending rows — the Reviewer name column keeps them distinct.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COLUMN DEFINITIONS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reviewer name   — Your full name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date            — Date of the observation (YYYY-MM-DD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tab             — Which app tab (Home, Data Input, QA/QC, Uncertainty, Correlations, Simulate, Sensitivity, IPCC Report, Resources, Definitions)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screen element  — The specific button, table, chart, or text that the comment relates to</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type            — Bug / Correction / Enhancement / General</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Severity        — Critical / High / Medium / Low</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Description     — What you observed or what the problem is</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suggested fix   — What the correct behaviour should be, or your proposed solution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status          — Leave blank; will be filled by the development team</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reviewer name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screen element / feature</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Severity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suggested fix / comment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type_def</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sev_def</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bug</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The tool crashes, produces wrong output, or behaves unexpectedly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Critical</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Must fix before any external release — calculation error or crash</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Something is factually incorrect — wrong equation, wrong IPCC reference, wrong number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Should fix before external release — significant usability or accuracy issue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enhancement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A feature that would make the tool more useful or easier to use</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Can fix in next iteration — minor issue that does not block use</t>
+  </si>
+  <si>
+    <t xml:space="preserve">General</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A general observation, question, or comment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nice to have — cosmetic or very minor improvement</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -192,22 +185,22 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <b/>
       <sz val="14"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <b/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <b/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <b/>
     </font>
   </fonts>
   <fills count="5">
@@ -242,13 +235,9 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
       <bottom style="thin">
         <color rgb="FF1B4332"/>
       </bottom>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -273,15 +262,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -563,173 +543,174 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A30"/>
-  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="100.7265625" customWidth="1"/>
+    <col min="1" max="1" width="100.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="6">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="7">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="8">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="9">
       <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="10">
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="11">
       <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="12">
       <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="13">
       <c r="A13" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="14">
       <c r="A14" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="15">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="16">
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:1" ht="29" x14ac:dyDescent="0.35">
+    <row r="18">
       <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="19">
       <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="20">
       <c r="A20" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="21">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="22">
       <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="23">
       <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="24">
       <c r="A24" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="25">
       <c r="A25" s="1"/>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="26">
       <c r="A26" s="1"/>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="27">
       <c r="A27" s="1"/>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="28">
       <c r="A28" s="1"/>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="29">
       <c r="A29" s="1"/>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="30">
       <c r="A30" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I50"/>
-  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="18.7265625" customWidth="1"/>
-    <col min="2" max="2" width="12.7265625" customWidth="1"/>
-    <col min="3" max="3" width="14.7265625" customWidth="1"/>
-    <col min="4" max="4" width="28.7265625" customWidth="1"/>
-    <col min="5" max="5" width="14.7265625" customWidth="1"/>
-    <col min="6" max="6" width="12.7265625" customWidth="1"/>
-    <col min="7" max="8" width="50.7265625" customWidth="1"/>
-    <col min="9" max="9" width="10.7265625" customWidth="1"/>
+    <col min="1" max="1" width="18.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="12.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="14.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="28.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="12.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="50.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="50.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="10.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" s="3" t="s">
         <v>23</v>
       </c>
@@ -758,7 +739,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2">
       <c r="A2" s="4"/>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
@@ -769,7 +750,7 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4">
       <c r="A4" s="4"/>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
@@ -780,7 +761,7 @@
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6">
       <c r="A6" s="4"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -791,7 +772,7 @@
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8">
       <c r="A8" s="4"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -802,7 +783,7 @@
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10">
       <c r="A10" s="4"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -813,7 +794,7 @@
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12">
       <c r="A12" s="4"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -824,7 +805,7 @@
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14">
       <c r="A14" s="4"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -835,7 +816,7 @@
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16">
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -846,7 +827,7 @@
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18">
       <c r="A18" s="4"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
@@ -857,7 +838,7 @@
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="20">
       <c r="A20" s="4"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -868,7 +849,7 @@
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="22">
       <c r="A22" s="4"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -879,7 +860,7 @@
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="24">
       <c r="A24" s="4"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -890,7 +871,7 @@
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="26">
       <c r="A26" s="4"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -901,7 +882,7 @@
       <c r="H26" s="4"/>
       <c r="I26" s="4"/>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="28">
       <c r="A28" s="4"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -912,7 +893,7 @@
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="30">
       <c r="A30" s="4"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -923,7 +904,7 @@
       <c r="H30" s="4"/>
       <c r="I30" s="4"/>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="32">
       <c r="A32" s="4"/>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -934,7 +915,7 @@
       <c r="H32" s="4"/>
       <c r="I32" s="4"/>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="34">
       <c r="A34" s="4"/>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -945,7 +926,7 @@
       <c r="H34" s="4"/>
       <c r="I34" s="4"/>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="36">
       <c r="A36" s="4"/>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -956,7 +937,7 @@
       <c r="H36" s="4"/>
       <c r="I36" s="4"/>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="38">
       <c r="A38" s="4"/>
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
@@ -967,7 +948,7 @@
       <c r="H38" s="4"/>
       <c r="I38" s="4"/>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="40">
       <c r="A40" s="4"/>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
@@ -978,7 +959,7 @@
       <c r="H40" s="4"/>
       <c r="I40" s="4"/>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="42">
       <c r="A42" s="4"/>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
@@ -989,7 +970,7 @@
       <c r="H42" s="4"/>
       <c r="I42" s="4"/>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="44">
       <c r="A44" s="4"/>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
@@ -1000,7 +981,7 @@
       <c r="H44" s="4"/>
       <c r="I44" s="4"/>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="46">
       <c r="A46" s="4"/>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -1011,7 +992,7 @@
       <c r="H46" s="4"/>
       <c r="I46" s="4"/>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="48">
       <c r="A48" s="4"/>
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>
@@ -1022,7 +1003,7 @@
       <c r="H48" s="4"/>
       <c r="I48" s="4"/>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="50">
       <c r="A50" s="4"/>
       <c r="B50" s="4"/>
       <c r="C50" s="4"/>
@@ -1034,47 +1015,61 @@
       <c r="I50" s="4"/>
     </row>
   </sheetData>
-  <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E200" xr:uid="{00000000-0002-0000-0100-000000000000}">
-      <formula1>"Bug,Correction,Enhancement,General"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F200" xr:uid="{00000000-0002-0000-0100-000001000000}">
-      <formula1>"Critical,High,Medium,Low"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C200" xr:uid="{00000000-0002-0000-0100-000002000000}">
-      <formula1>"Home,Data Input,QA/QC,Uncertainty,Correlations,Simulate,Sensitivity,IPCC Report,Resources,Definitions,General (whole app)"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"Bug,Correction,Enhancement,General"</xm:f>
+          </x14:formula1>
+          <xm:sqref>E2:E200</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"Critical,High,Medium,Low"</xm:f>
+          </x14:formula1>
+          <xm:sqref>F2:F200</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"Home,Data Input,QA/QC,Uncertainty,Correlations,Simulate,Sensitivity,IPCC Report,Resources,Definitions,General (whole app)"</xm:f>
+          </x14:formula1>
+          <xm:sqref>C2:C200</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="16.7265625" customWidth="1"/>
-    <col min="2" max="2" width="14.7265625" customWidth="1"/>
-    <col min="3" max="4" width="55.7265625" customWidth="1"/>
+    <col min="1" max="1" width="16.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="55.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="14.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="55.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" s="6" t="s">
         <v>27</v>
       </c>
       <c r="B1" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" s="6" t="s">
         <v>28</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>32</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="2">
       <c r="A2" s="5" t="s">
         <v>34</v>
       </c>
@@ -1088,7 +1083,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="3">
       <c r="A3" s="5" t="s">
         <v>38</v>
       </c>
@@ -1102,7 +1097,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4">
       <c r="A4" s="5" t="s">
         <v>42</v>
       </c>
@@ -1116,7 +1111,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5">
       <c r="A5" s="5" t="s">
         <v>46</v>
       </c>
@@ -1132,31 +1127,11 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="03e19825-731a-404b-84c3-310fff85d1a8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="a675dd88-c1ff-478a-b60f-ff004313760b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006AAA32E7549EE6449AC68337FF671C5A" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5b725368af9e92254b31af2044252fac">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="03e19825-731a-404b-84c3-310fff85d1a8" xmlns:ns3="a675dd88-c1ff-478a-b60f-ff004313760b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="de1faf0135fd982ba30b50c3b754e7cb" ns2:_="" ns3:_="">
     <xsd:import namespace="03e19825-731a-404b-84c3-310fff85d1a8"/>
@@ -1357,40 +1332,34 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="03e19825-731a-404b-84c3-310fff85d1a8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="a675dd88-c1ff-478a-b60f-ff004313760b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F02E372A-8436-4AE8-8051-0E802A6948C5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="03e19825-731a-404b-84c3-310fff85d1a8"/>
-    <ds:schemaRef ds:uri="a675dd88-c1ff-478a-b60f-ff004313760b"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{408BF082-2FAA-468F-9D7C-6476A9B49E30}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{41836187-7F0B-4708-A329-BA861C1C799B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AB335A62-4A64-4827-A761-73BA305334BC}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FB5A6083-7723-4AF9-AB8F-EC8511598099}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="03e19825-731a-404b-84c3-310fff85d1a8"/>
-    <ds:schemaRef ds:uri="a675dd88-c1ff-478a-b60f-ff004313760b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{32F7BFCE-A837-4055-8148-60C60A336225}"/>
 </file>
</xml_diff>